<commit_message>
Modulo iscrizioni: data e prezzo in bianco, scelte in linea, pagamento in loco
</commit_message>
<xml_diff>
--- a/MODULO-iscrizioni-AGGIORNATO.xlsx
+++ b/MODULO-iscrizioni-AGGIORNATO.xlsx
@@ -525,7 +525,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
@@ -1189,7 +1189,7 @@
       <c r="F19" s="7" t="inlineStr"/>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>da saldare sul posto</t>
+          <t>Pagamento in Loco</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1444,11 +1444,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="98" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Sequenza di comparsa. Procedere per decine (10, 20, 30...) per inserire voci intermedie.</t>
+          <t>Sequenza di comparsa. Procedere per decine (10, 20, 30...).</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Nome tecnico del campo. NON modificare gli ID esistenti. Vuoto per titoli e testi informativi.</t>
+          <t>Nome tecnico del campo. NON modificare gli ID esistenti.</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Il testo della domanda o del titolo, come apparira sul sito.</t>
+          <t>Il testo della domanda o del titolo.</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Sottotitolo o testo di aiuto mostrato sotto la domanda.</t>
+          <t>Sottotitolo o testo di aiuto sotto la domanda.</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Un NUMERO concorre al totale del bonifico. Un TESTO (es. da saldare sul posto) viene solo mostrato, senza addebito.</t>
+          <t>Un NUMERO concorre al totale del bonifico. Un TESTO (es. Pagamento in Loco) viene solo mostrato, senza addebito.</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>NO nasconde la voce dal modulo senza cancellarla.</t>
+          <t>NO nasconde la voce senza cancellarla.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       <c r="A18" s="15" t="inlineStr"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Perche funzioni, l Etichetta deve iniziare con la data. Esempio:</t>
+          <t>L Etichetta deve iniziare con la data. Esempio:</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       <c r="A20" s="15" t="inlineStr"/>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>La data compare una sola volta come testata del gruppo, non nella singola voce.</t>
+          <t>La data compare una sola volta come testata del gruppo.</t>
         </is>
       </c>
     </row>
@@ -1650,60 +1650,28 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>ESEMPI</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr"/>
+          <t>AVVERTENZA</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Il foglio deve chiamarsi esattamente Modulo.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Variare un prezzo</t>
-        </is>
-      </c>
+      <c r="A23" s="15" t="inlineStr"/>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Modificare la colonna Prezzo: totale sul sito ed email si aggiornano da soli.</t>
+          <t>Aggiungendo o togliendo domande cambiano le colonne del foglio Iscrizioni:</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Sospendere una voce</t>
-        </is>
-      </c>
+      <c r="A24" s="15" t="inlineStr"/>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Scrivere NO nella colonna Attiva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Aggiungere un attivita</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Nuova riga con Ordine intermedio, ID nuovo, Tipo sino, prezzo, SI in Obbligatoria e Attiva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr"/>
-      <c r="B26" s="11" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>AVVERTENZA</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Il foglio deve chiamarsi esattamente Modulo. Le risposte sono scritte nel foglio Iscrizioni.</t>
+          <t>in tal caso eliminare il foglio Iscrizioni vuoto ed eseguire di nuovo setup.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Attivita su tre colonne: orario evidenziato, costo in colonna propria, selezione piu chiara
</commit_message>
<xml_diff>
--- a/MODULO-iscrizioni-AGGIORNATO.xlsx
+++ b/MODULO-iscrizioni-AGGIORNATO.xlsx
@@ -523,7 +523,7 @@
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -949,7 +949,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Galleria Subalpina 16, 10123 Torino — costo a carico del partecipante</t>
+          <t>Ristorante Arcadia — Galleria Subalpina 16, 10123 Torino</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>NH Carlina, P.za Carlo Emanuele II 15 — Centralino Club, Via delle Rosine 16, Torino — costo complessivo a carico del partecipante</t>
+          <t>NH Carlina, P.za Carlo Emanuele II 15 — Centralino Club, Via delle Rosine 16, Torino</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Sede da definire — costo a carico del partecipante</t>
+          <t>Sede da definire</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Sede da definire — costo a carico del partecipante, da regolare sul posto: NON è compreso nel bonifico</t>
+          <t>Sede da definire — da saldare sul posto, non compreso nel bonifico</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr"/>
@@ -1444,11 +1444,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Il testo della domanda o del titolo.</t>
+          <t>Il testo della domanda. Per le attivita: DATA, ore ORARIO - Titolo attivita</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Sottotitolo o testo di aiuto sotto la domanda.</t>
+          <t>Sede e note. Non serve ripetere il costo: viene mostrato nel riquadro a fianco.</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Un NUMERO concorre al totale del bonifico. Un TESTO (es. Pagamento in Loco) viene solo mostrato, senza addebito.</t>
+          <t>Un NUMERO concorre al totale del bonifico. Un TESTO (es. Pagamento in Loco) viene solo mostrato.</t>
         </is>
       </c>
     </row>
@@ -1610,20 +1610,16 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>RAGGRUPPAMENTO PER DATA</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Le attivita di tipo "sino" sono raggruppate automaticamente per data.</t>
-        </is>
-      </c>
+          <t>COME APPARE UN ATTIVITA</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr"/>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>L Etichetta deve iniziare con la data. Esempio:</t>
+          <t>Il modulo dispone ogni attivita su tre colonne:</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1627,7 @@
       <c r="A19" s="15" t="inlineStr"/>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>23 ottobre 2026, ore 10:00 - Consiglio Nazionale Giovani GIE ANCE</t>
+          <t>1) orario e titolo   2) riquadro del costo   3) Si partecipo / No non partecipo</t>
         </is>
       </c>
     </row>
@@ -1639,37 +1635,81 @@
       <c r="A20" s="15" t="inlineStr"/>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>La data compare una sola volta come testata del gruppo.</t>
+          <t>L orario viene estratto dall Etichetta ed evidenziato in arancione.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr"/>
-      <c r="B21" s="11" t="inlineStr"/>
+      <c r="A21" s="15" t="inlineStr"/>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Le attivita sono raggruppate automaticamente per data.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>AVVERTENZA</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Il foglio deve chiamarsi esattamente Modulo.</t>
-        </is>
-      </c>
+      <c r="A22" s="12" t="inlineStr"/>
+      <c r="B22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr"/>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Aggiungendo o togliendo domande cambiano le colonne del foglio Iscrizioni:</t>
-        </is>
-      </c>
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>CAUSALE DEL BONIFICO</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr"/>
       <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Generata cosi: COGNOME NOME CONVEGNO AN 2026 seguito dalle sigle delle attivita pagate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr"/>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>La sigla e la prima parola significativa del titolo piu il giorno. Esempi: CENA22, APERITIVO23, VISITA24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr"/>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Per cambiare una sigla, modificare la prima parola del titolo nell Etichetta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr"/>
+      <c r="B27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>AVVERTENZA</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Il foglio deve chiamarsi esattamente Modulo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Aggiungendo o togliendo domande cambiano le colonne del foglio Iscrizioni:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr"/>
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>in tal caso eliminare il foglio Iscrizioni vuoto ed eseguire di nuovo setup.</t>
         </is>

</xml_diff>